<commit_message>
Corte: se agregan Lecturas 1 y 2 (Discussions)
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-05sep.xlsx
+++ b/calificaciones/P00-S02-corte-05sep.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="P00 y S02" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="P00 · S02 · Lecturas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Cómo-entregar-p00" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -87,12 +87,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFCDD2"/>
+        <fgColor rgb="00F2F5F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F5F9"/>
+        <fgColor rgb="00FFCDD2"/>
       </patternFill>
     </fill>
     <fill>
@@ -139,14 +139,14 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -526,34 +526,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SD 1959-2 · Tarea de Git (P00) y adelanto de la práctica Docker (S02) · por número de cuenta</t>
+          <t>SD 1959-2 · Corte: tarea de Git (P00), práctica Docker (S02) y Lecturas 1-2 · por número de cuenta</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Revisión: 05-sep-2026, 06:12 · La entrega es en TU rama (entregas_apellido_nombre o tu s02-…); el PR va al FINAL del curso.</t>
+          <t>Revisión: 05-sep-2026, 06:39 · La entrega es en TU rama entregas_apellido_nombre (push = entrega); el PR va al FINAL del curso.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>P00: entregas/apellido_nombre/p00/prueba.txt en tu rama.   S02: la práctica de Docker (Dockerfile + evidencia.md + index.html) — aún no es obligatoria; ✓/parcial es adelanto.</t>
+          <t>P00: entregas/apellido_nombre/p00/prueba.txt.  S02: práctica Docker (aún no obligatoria; ✓/parcial es adelanto).  L1: opcional.  L2: 2 preguntas + 1 hallazgo en la Discussion #2.  ¿? = confirma tu usuario en clase.</t>
         </is>
       </c>
     </row>
@@ -579,6 +581,16 @@
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>L1 (opc.)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
@@ -603,7 +615,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>falta la Lectura 2 en Discussions</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -619,12 +645,22 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>sin actividad en el repositorio</t>
         </is>
@@ -651,9 +687,15 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>PR abierto: el PR va al final del curso</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -669,12 +711,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>falta la Lectura 2 en Discussions</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -695,7 +751,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -711,12 +777,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr"/>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -732,14 +808,24 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>sin actividad en el repositorio</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>¿?</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>confirma en clase si participaste en la Lectura 2</t>
         </is>
       </c>
     </row>
@@ -764,7 +850,17 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>s02 incompleta (falta Dockerfile/evidencia) · PR abierto</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>s02 incompleta (falta Dockerfile/evidencia)</t>
         </is>
       </c>
     </row>
@@ -782,12 +878,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr"/>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -803,14 +909,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>la rama debe llamarse entregas_apellido_nombre · PR abierto</t>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>usa tu rama entregas_ nueva</t>
         </is>
       </c>
     </row>
@@ -835,7 +951,17 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>falta el p00 (ver hoja Cómo-entregar-p00) · PR abierto</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>falta el p00 (hoja Cómo-entregar-p00) y la Lectura 2</t>
         </is>
       </c>
     </row>
@@ -860,7 +986,17 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>falta el p00 · s02 incompleta · PR abierto</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>falta el p00 · s02 incompleta</t>
         </is>
       </c>
     </row>
@@ -878,14 +1014,24 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>sin actividad en el repositorio</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>¿?</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>confirma en clase tu usuario de GitHub (¿participaste en la Lectura 2?)</t>
         </is>
       </c>
     </row>
@@ -903,12 +1049,22 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>sin actividad en el repositorio</t>
         </is>
@@ -928,12 +1084,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>falta la Lectura 2 en Discussions</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
@@ -949,12 +1119,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -970,12 +1150,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>falta la Lectura 2 en Discussions</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -998,7 +1192,17 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>tu carpeta va con apellido_nombre completo · PR abierto</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>tu carpeta va con apellido_nombre completo · falta la Lectura 2</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1220,22 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
         <is>
           <t>sin actividad en el repositorio</t>
         </is>
@@ -1041,12 +1255,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr"/>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>falta la Lectura 2 en Discussions</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
@@ -1069,7 +1297,17 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>falta el p00 (ver hoja Cómo-entregar-p00) · PR abierto</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>falta el p00 (hoja Cómo-entregar-p00)</t>
         </is>
       </c>
     </row>
@@ -1094,9 +1332,15 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>PR abierto</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -1117,9 +1361,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>tu rama está vacía: si te atoraste en el lab, acércate — lo resolvemos rápido</t>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>tu rama está vacía: si te atoraste en el lab, acércate — tus lecturas van muy bien</t>
         </is>
       </c>
     </row>
@@ -1137,14 +1391,24 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>sin actividad en el repositorio</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>¿?</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>confirma en clase si participaste en la Lectura 2</t>
         </is>
       </c>
     </row>
@@ -1162,12 +1426,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr"/>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
@@ -1183,14 +1457,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>PR abierto: el PR va al final del curso</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>falta la Lectura 2 en Discussions</t>
         </is>
       </c>
     </row>
@@ -1208,12 +1492,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr"/>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
@@ -1229,16 +1523,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>PR abierto: el PR va al final del curso</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -1261,9 +1561,15 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>PR abierto</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
@@ -1279,12 +1585,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
         <is>
           <t>tu carpeta va en minúsculas: apellido_nombre</t>
         </is>
@@ -1304,12 +1620,22 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
         <is>
           <t>sin actividad en el repositorio</t>
         </is>
@@ -1334,9 +1660,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>PR abierto</t>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>hiciste la L1 (opcional) pero falta la Lectura 2</t>
         </is>
       </c>
     </row>
@@ -1354,12 +1690,22 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D38" s="9" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="inlineStr">
         <is>
           <t>sin actividad en el repositorio</t>
         </is>
@@ -1386,7 +1732,17 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>tienes dos ramas: quédate con la entregas_ y cierra el PR de la vieja</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>falta la Lectura 2 en Discussions</t>
         </is>
       </c>
     </row>
@@ -1404,12 +1760,22 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
         <is>
           <t>sin actividad en el repositorio</t>
         </is>
@@ -1436,9 +1802,15 @@
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>PR abierto</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
@@ -1454,12 +1826,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D42" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr"/>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n">
@@ -1482,7 +1864,17 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>falta el p00 (ver hoja Cómo-entregar-p00)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>falta el p00 (hoja Cómo-entregar-p00)</t>
         </is>
       </c>
     </row>
@@ -1500,14 +1892,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>PR abierto: el PR va al final del curso</t>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>muy bien: L1 y L2 completas</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1934,17 @@
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>falta el p00 (ver hoja Cómo-entregar-p00) · PR abierto</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>falta el p00 (hoja Cómo-entregar-p00)</t>
         </is>
       </c>
     </row>
@@ -1555,9 +1967,19 @@
           <t>parcial</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>s02 incompleta: falta evidencia.md</t>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>s02 incompleta: falta evidencia.md · lecturas muy bien</t>
         </is>
       </c>
     </row>
@@ -1582,7 +2004,17 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>falta el p00 (ver hoja Cómo-entregar-p00)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>falta el p00 (hoja Cómo-entregar-p00)</t>
         </is>
       </c>
     </row>
@@ -1600,12 +2032,22 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D48" s="9" t="inlineStr">
+      <c r="D48" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
         <is>
           <t>sin actividad en el repositorio</t>
         </is>
@@ -1614,7 +2056,7 @@
     <row r="50">
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>Resumen: P00 entregada 26/43 · con rama pero sin p00: 7 · sin nada: 10 · Docker S02 completa: 13, parcial: 4</t>
+          <t>Resumen: P00 26/43 · S02 completa 13, parcial 4 · L1 (opcional) 5 · L2 entregada 23 confirmadas + 2 por confirmar</t>
         </is>
       </c>
     </row>
@@ -1630,10 +2072,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="76" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1647,7 +2089,7 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>Donde diga tu_apellido_nombre o TU-RAMA, escribe TUS nombres reales (tu rama es entregas_apellido_nombre, o tu s02-… si ya la tenías).</t>
+          <t>Tu rama entregas_apellido_nombre YA existe (te la creamos desde tu rama del lab). Donde diga tu_apellido_nombre, escribe TUS nombres reales.</t>
         </is>
       </c>
     </row>
@@ -1666,103 +2108,91 @@
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>git checkout main</t>
+          <t>git fetch origin</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>párate en main</t>
+          <t>entérate de las ramas nuevas (incluida la tuya)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git checkout entregas_tu_apellido_nombre</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>trae lo más nuevo</t>
+          <t>cámbiate a TU rama del semestre</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>git checkout TU-RAMA</t>
+          <t>mkdir -p entregas/tu_apellido_nombre/p00</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>cámbiate a tu rama (o créala: git checkout -b entregas_tu_apellido_nombre)</t>
+          <t>crea tu carpeta de la p00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>mkdir -p entregas/tu_apellido_nombre/p00</t>
+          <t>echo "Prueba - Nombre y Apellido!" &gt; entregas/tu_apellido_nombre/p00/prueba.txt</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>crea tu carpeta de la p00</t>
+          <t>el archivo de prueba — escribe TU nombre</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>echo "Prueba - Nombre y Apellido!" &gt; entregas/tu_apellido_nombre/p00/prueba.txt</t>
+          <t>git add entregas/tu_apellido_nombre/p00</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>el archivo de prueba — escribe TU nombre</t>
+          <t>prepara el archivo</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/p00</t>
+          <t>git commit -m "P00: prueba de git"</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>prepara el archivo</t>
+          <t>guárdalo con mensaje claro</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>git commit -m "P00: prueba de git"</t>
+          <t>git push -u origin entregas_tu_apellido_nombre</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>guárdalo con mensaje claro</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>git push origin TU-RAMA</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>súbelo a GitHub — y listo, NO abras PR: ese va al final del curso</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>En esa MISMA rama irán TODAS tus entregas individuales del semestre.</t>
+          <t>súbelo — y listo, NO abras PR: ese va al final del curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>En esa MISMA rama van TODAS tus entregas individuales del semestre. Las lecturas van en Discussions cada semana.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corte actualizado: p00 y s02 del 05-sep, lecturas tarde adjudicables
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-05sep.xlsx
+++ b/calificaciones/P00-S02-corte-05sep.xlsx
@@ -531,11 +531,11 @@
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="72" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,14 +548,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Revisión: 05-sep-2026, 06:39 · La entrega es en TU rama entregas_apellido_nombre (push = entrega); el PR va al FINAL del curso.</t>
+          <t>Revisión: 05-sep-2026, 09:36 · La entrega es en TU rama entregas_apellido_nombre (push = entrega); el PR va al FINAL del curso.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>P00: entregas/apellido_nombre/p00/prueba.txt.  S02: práctica Docker (aún no obligatoria; ✓/parcial es adelanto).  L1: opcional.  L2: 2 preguntas + 1 hallazgo en la Discussion #2.  ¿? = confirma tu usuario en clase.</t>
+          <t>P00: entregas/apellido_nombre/p00/prueba.txt.  S02: práctica Docker (aún no obligatoria; ✓/parcial es adelanto).  L1: opcional.  L2: Discussion #2 (cierre sábado 06:59; 'tarde' = entró después y se adjudica).  ¿? = confirma tu usuario en clase.</t>
         </is>
       </c>
     </row>
@@ -924,11 +924,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>usa tu rama entregas_ nueva</t>
-        </is>
-      </c>
+      <c r="G15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -939,9 +935,9 @@
           <t>117003136</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -961,7 +957,7 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>falta el p00 (hoja Cómo-entregar-p00) y la Lectura 2</t>
+          <t>falta la Lectura 2 en Discussions</t>
         </is>
       </c>
     </row>
@@ -974,14 +970,14 @@
           <t>321058526</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>parcial</t>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -996,7 +992,7 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>falta el p00 · s02 incompleta</t>
+          <t>archivos .py extra en tu p00: solo va prueba.txt (menor)</t>
         </is>
       </c>
     </row>
@@ -1009,14 +1005,14 @@
           <t>320046045</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>parcial</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
@@ -1024,14 +1020,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>¿?</t>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>confirma en clase tu usuario de GitHub (¿participaste en la Lectura 2?)</t>
+          <t>tu prueba va en p00/prueba.txt (no en s02/) · usa tu rama entregas_guerrero_uriel · falta el contenido Docker del s02</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1233,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>sin actividad en el repositorio</t>
+          <t>tu rama existe pero está vacía: sube tu p00 (hoja Cómo-entregar-p00)</t>
         </is>
       </c>
     </row>
@@ -1255,9 +1251,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -1351,9 +1347,9 @@
           <t>320094187</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>parcial</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -1373,7 +1369,7 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>tu rama está vacía: si te atoraste en el lab, acércate — tus lecturas van muy bien</t>
+          <t>tu prueba.txt quedó en s02/: muévela a p00/prueba.txt · el contenido Docker del s02 sigue pendiente — acércate, tus lecturas van muy bien</t>
         </is>
       </c>
     </row>
@@ -1457,9 +1453,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -1474,7 +1470,7 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>falta la Lectura 2 en Discussions</t>
+          <t>renombra 'S02 Lab Docker.md' a evidencia.md (menor) · falta la Lectura 2</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1633,7 @@
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>sin actividad en el repositorio</t>
+          <t>acepta tu invitación al repositorio (github.com/notifications)</t>
         </is>
       </c>
     </row>
@@ -1665,14 +1661,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>tarde</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>hiciste la L1 (opcional) pero falta la Lectura 2</t>
+          <t>tu Lectura 2 entró a las 07:28, después del cierre (06:59): se revisará si cuenta</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1703,7 @@
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>sin actividad en el repositorio</t>
+          <t>acepta tu invitación nueva al repositorio</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1738,7 @@
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>falta la Lectura 2 en Discussions</t>
+          <t>s02 incompleta (solo hello.py) · falta la Lectura 2</t>
         </is>
       </c>
     </row>
@@ -1777,7 +1773,7 @@
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>sin actividad en el repositorio</t>
+          <t>acepta tu invitación nueva al repositorio</t>
         </is>
       </c>
     </row>
@@ -1852,9 +1848,9 @@
           <t>317042333</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
@@ -1872,11 +1868,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G43" s="9" t="inlineStr">
-        <is>
-          <t>falta el p00 (hoja Cómo-entregar-p00)</t>
-        </is>
-      </c>
+      <c r="G43" s="9" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -1922,9 +1914,9 @@
           <t>318259624</t>
         </is>
       </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -1942,11 +1934,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G45" s="9" t="inlineStr">
-        <is>
-          <t>falta el p00 (hoja Cómo-entregar-p00)</t>
-        </is>
-      </c>
+      <c r="G45" s="9" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
@@ -2042,21 +2030,21 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>tarde</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>sin actividad en el repositorio</t>
+          <t>tu Lectura 2 entró a las 07:00, un minuto después del cierre: se revisará · falta todo el repo (p00)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>Resumen: P00 26/43 · S02 completa 13, parcial 4 · L1 (opcional) 5 · L2 entregada 23 confirmadas + 2 por confirmar</t>
+          <t>Resumen: P00 30/43 (+2 parciales por carpeta) · S02 completa 16, parcial 3 · L1 (opcional) 5 · L2: 24 a tiempo + 2 tarde + 1 por confirmar</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2077,7 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>Tu rama entregas_apellido_nombre YA existe (te la creamos desde tu rama del lab). Donde diga tu_apellido_nombre, escribe TUS nombres reales.</t>
+          <t>Tu rama entregas_apellido_nombre YA existe (si tienes cualquier actividad previa). Donde diga tu_apellido_nombre, escribe TUS nombres reales.</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2113,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>cámbiate a TU rama del semestre</t>
+          <t>cámbiate a TU rama del semestre (si no existe: git checkout -b entregas_tu_apellido_nombre)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Politica de tiempos: labs en tiempo hasta el domingo, tarde no penaliza (solo tendencia); lecturas sabado 06:59 / tarde hasta domingo
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-05sep.xlsx
+++ b/calificaciones/P00-S02-corte-05sep.xlsx
@@ -548,14 +548,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Revisión: 05-sep-2026, 09:36 · La entrega es en TU rama entregas_apellido_nombre (push = entrega); el PR va al FINAL del curso.</t>
+          <t>Revisión: 05-sep-2026, 10:44 · La entrega es en TU rama entregas_apellido_nombre (push = entrega); el PR va al FINAL del curso.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>P00: entregas/apellido_nombre/p00/prueba.txt.  S02: práctica Docker (aún no obligatoria; ✓/parcial es adelanto).  L1: opcional.  L2: Discussion #2 (cierre sábado 06:59; 'tarde' = entró después y se adjudica).  ¿? = confirma tu usuario en clase.</t>
+          <t>P00: entregas/apellido_nombre/p00/prueba.txt.  S02: práctica Docker (aún no obligatoria; ✓/parcial es adelanto).  L1: opcional.  L2: Discussion #2 (en tiempo hasta sáb 06:59 · tarde hasta el domingo — tarde no penaliza, se registra para la tendencia).  ¿? = confirma tu usuario en clase.</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>tu Lectura 2 entró a las 07:28, después del cierre (06:59): se revisará si cuenta</t>
+          <t>tu Lectura 2 entró tarde (07:28): cuenta, y queda en tu tendencia de entregas</t>
         </is>
       </c>
     </row>
@@ -2037,14 +2037,14 @@
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>tu Lectura 2 entró a las 07:00, un minuto después del cierre: se revisará · falta todo el repo (p00)</t>
+          <t>tu Lectura 2 entró tarde (07:00): cuenta, queda en tu tendencia · falta todo el repo (p00)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>Resumen: P00 30/43 (+2 parciales por carpeta) · S02 completa 16, parcial 3 · L1 (opcional) 5 · L2: 24 a tiempo + 2 tarde + 1 por confirmar</t>
+          <t>Resumen: P00 30/43 (+2 parciales por carpeta) · S02 completa 16, parcial 3 · L1 (opcional) 5 · L2: 24 en tiempo + 2 tarde (válidas) + 1 por confirmar</t>
         </is>
       </c>
     </row>

</xml_diff>